<commit_message>
Update price table: new daily rates and OT multipliers 1.34/1.67
翻譯 3500, 工安 3500, 工安Leader 3600; OT and holiday hourly rates
recomputed from daily wage; add per-person rate notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyDty1wfvKkCTcRnVVfnEm
</commit_message>
<xml_diff>
--- a/output/2027點工單價_簡表.xlsx
+++ b/output/2027點工單價_簡表.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -549,19 +549,19 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3400</v>
+        <v>3500</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>565</v>
+        <v>586</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>706</v>
+        <v>731</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>706</v>
+        <v>731</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>850</v>
+        <v>875</v>
       </c>
     </row>
     <row r="7">
@@ -576,19 +576,19 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3300</v>
+        <v>3500</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>548.625</v>
+        <v>586</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>684.75</v>
+        <v>731</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>684.75</v>
+        <v>731</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>825</v>
+        <v>875</v>
       </c>
     </row>
     <row r="8">
@@ -603,19 +603,19 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>3400</v>
+        <v>3600</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>565</v>
+        <v>603</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>706</v>
+        <v>752</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>706</v>
+        <v>752</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>850</v>
+        <v>900</v>
       </c>
     </row>
     <row r="9">
@@ -633,13 +633,13 @@
         <v>3800</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>950</v>
@@ -660,13 +660,13 @@
         <v>4000</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>830</v>
+        <v>835</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>830</v>
+        <v>835</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>1000</v>
@@ -687,13 +687,13 @@
         <v>3500</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>875</v>
@@ -714,13 +714,13 @@
         <v>3800</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="G12" s="4" t="n">
         <v>950</v>
@@ -741,13 +741,13 @@
         <v>3800</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="G13" s="4" t="n">
         <v>950</v>
@@ -785,6 +785,20 @@
       <c r="A19" t="inlineStr">
         <is>
           <t>4. 春節紅包:1,000 元(春節出勤,日班/夜班皆適用)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>5. 平日加班倍率:2H內 ×1.34、3H以上 ×1.67(以日薪÷8 為時薪計算,四捨五入至整數)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>6. 指定人員單價:琬婷 → 比照工安Leader;振揮 → 比照CS On-Site leader。</t>
         </is>
       </c>
     </row>

</xml_diff>